<commit_message>
Starten på anden uge i Juli. 2 uger til at jeg vil have bacheloren færdig
</commit_message>
<xml_diff>
--- a/7. Semester/Bachelor clean/results.xlsx
+++ b/7. Semester/Bachelor clean/results.xlsx
@@ -13,7 +13,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="146" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="126" uniqueCount="7">
+  <si>
+    <t>Typer</t>
+  </si>
   <si>
     <t>nf_max</t>
   </si>
@@ -31,12 +34,6 @@
   </si>
   <si>
     <t>volFrac_min</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Typer</t>
   </si>
 </sst>
 </file>
@@ -96,25 +93,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Går ind i sidste uge af bacheloropgaveskrivningen, og mangler lidt arbejde endnu
</commit_message>
<xml_diff>
--- a/7. Semester/Bachelor clean/results.xlsx
+++ b/7. Semester/Bachelor clean/results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="126" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="161" uniqueCount="7">
   <si>
     <t>Typer</t>
   </si>
@@ -119,22 +119,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>21.370999999999999</v>
+        <v>3.419</v>
       </c>
       <c r="C2" s="0">
-        <v>8.1489999999999991</v>
+        <v>2.2450000000000001</v>
       </c>
       <c r="D2" s="0">
-        <v>0.39200000000000002</v>
+        <v>1.0109999999999999</v>
       </c>
       <c r="E2" s="0">
-        <v>1.2729999999999999</v>
+        <v>1.272</v>
       </c>
       <c r="F2" s="0">
-        <v>0.96899999999999997</v>
+        <v>0.93799999999999994</v>
       </c>
       <c r="G2" s="0">
-        <v>-0.503</v>
+        <v>-0.58899999999999997</v>
       </c>
     </row>
     <row r="3">
@@ -142,22 +142,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>13.417</v>
+        <v>3.4249999999999998</v>
       </c>
       <c r="C3" s="0">
-        <v>5.8289999999999997</v>
+        <v>2.3279999999999998</v>
       </c>
       <c r="D3" s="0">
-        <v>0.36899999999999999</v>
+        <v>1.0209999999999999</v>
       </c>
       <c r="E3" s="0">
         <v>1.26</v>
       </c>
       <c r="F3" s="0">
-        <v>0.90500000000000003</v>
+        <v>0.90600000000000003</v>
       </c>
       <c r="G3" s="0">
-        <v>-0.51800000000000002</v>
+        <v>-0.63600000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -165,22 +165,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>6.9349999999999996</v>
+        <v>3.4079999999999999</v>
       </c>
       <c r="C4" s="0">
-        <v>3.1949999999999998</v>
+        <v>2.113</v>
       </c>
       <c r="D4" s="0">
-        <v>0.105</v>
+        <v>1.006</v>
       </c>
       <c r="E4" s="0">
         <v>1.204</v>
       </c>
       <c r="F4" s="0">
-        <v>0.56899999999999995</v>
+        <v>0.51500000000000001</v>
       </c>
       <c r="G4" s="0">
-        <v>-0.63</v>
+        <v>-0.63400000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -188,22 +188,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>5.4980000000000002</v>
+        <v>3.4239999999999999</v>
       </c>
       <c r="C5" s="0">
-        <v>2.5059999999999998</v>
+        <v>2.161</v>
       </c>
       <c r="D5" s="0">
-        <v>0.044999999999999998</v>
+        <v>1.0009999999999999</v>
       </c>
       <c r="E5" s="0">
-        <v>1.1619999999999999</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="F5" s="0">
-        <v>0.52400000000000002</v>
+        <v>0.50600000000000001</v>
       </c>
       <c r="G5" s="0">
-        <v>-0.63800000000000001</v>
+        <v>-0.63900000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -211,22 +211,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>6.3789999999999996</v>
+        <v>3.423</v>
       </c>
       <c r="C6" s="0">
-        <v>3.5369999999999999</v>
+        <v>2.1320000000000001</v>
       </c>
       <c r="D6" s="0">
-        <v>0.091999999999999998</v>
+        <v>1.002</v>
       </c>
       <c r="E6" s="0">
         <v>1.1910000000000001</v>
       </c>
       <c r="F6" s="0">
-        <v>0.68300000000000005</v>
+        <v>0.56599999999999995</v>
       </c>
       <c r="G6" s="0">
-        <v>-0.63200000000000001</v>
+        <v>-0.63800000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -234,22 +234,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>7.2830000000000004</v>
+        <v>3.4239999999999999</v>
       </c>
       <c r="C7" s="0">
-        <v>3.2240000000000002</v>
+        <v>2.2360000000000002</v>
       </c>
       <c r="D7" s="0">
-        <v>0.14799999999999999</v>
+        <v>1.117</v>
       </c>
       <c r="E7" s="0">
         <v>1.2110000000000001</v>
       </c>
       <c r="F7" s="0">
-        <v>0.623</v>
+        <v>0.56299999999999994</v>
       </c>
       <c r="G7" s="0">
-        <v>-0.62</v>
+        <v>-0.622</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bachelor afleveret, nu bare forsvar tilbage
</commit_message>
<xml_diff>
--- a/7. Semester/Bachelor clean/results.xlsx
+++ b/7. Semester/Bachelor clean/results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="161" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="259" uniqueCount="7">
   <si>
     <t>Typer</t>
   </si>
@@ -119,22 +119,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>3.419</v>
+        <v>21.370999999999999</v>
       </c>
       <c r="C2" s="0">
-        <v>2.2450000000000001</v>
+        <v>7.3879999999999999</v>
       </c>
       <c r="D2" s="0">
-        <v>1.0109999999999999</v>
+        <v>0.091999999999999998</v>
       </c>
       <c r="E2" s="0">
-        <v>1.272</v>
+        <v>1.2729999999999999</v>
       </c>
       <c r="F2" s="0">
-        <v>0.93799999999999994</v>
+        <v>0.93999999999999995</v>
       </c>
       <c r="G2" s="0">
-        <v>-0.58899999999999997</v>
+        <v>-0.63200000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -142,19 +142,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>3.4249999999999998</v>
+        <v>13.417</v>
       </c>
       <c r="C3" s="0">
-        <v>2.3279999999999998</v>
+        <v>5.3049999999999997</v>
       </c>
       <c r="D3" s="0">
-        <v>1.0209999999999999</v>
+        <v>0.068000000000000005</v>
       </c>
       <c r="E3" s="0">
         <v>1.26</v>
       </c>
       <c r="F3" s="0">
-        <v>0.90600000000000003</v>
+        <v>0.85299999999999998</v>
       </c>
       <c r="G3" s="0">
         <v>-0.63600000000000001</v>
@@ -165,19 +165,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>3.4079999999999999</v>
+        <v>6.9340000000000002</v>
       </c>
       <c r="C4" s="0">
-        <v>2.113</v>
+        <v>3.0619999999999998</v>
       </c>
       <c r="D4" s="0">
-        <v>1.006</v>
+        <v>0.085000000000000006</v>
       </c>
       <c r="E4" s="0">
         <v>1.204</v>
       </c>
       <c r="F4" s="0">
-        <v>0.51500000000000001</v>
+        <v>0.56699999999999995</v>
       </c>
       <c r="G4" s="0">
         <v>-0.63400000000000001</v>
@@ -188,22 +188,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>3.4239999999999999</v>
+        <v>5.4980000000000002</v>
       </c>
       <c r="C5" s="0">
-        <v>2.161</v>
+        <v>2.29</v>
       </c>
       <c r="D5" s="0">
-        <v>1.0009999999999999</v>
+        <v>0.014999999999999999</v>
       </c>
       <c r="E5" s="0">
-        <v>1.1579999999999999</v>
+        <v>1.1619999999999999</v>
       </c>
       <c r="F5" s="0">
-        <v>0.50600000000000001</v>
+        <v>0.45700000000000002</v>
       </c>
       <c r="G5" s="0">
-        <v>-0.63900000000000001</v>
+        <v>-0.64000000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -211,19 +211,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>3.423</v>
+        <v>6.3869999999999996</v>
       </c>
       <c r="C6" s="0">
-        <v>2.1320000000000001</v>
+        <v>3.5110000000000001</v>
       </c>
       <c r="D6" s="0">
-        <v>1.002</v>
+        <v>0.053999999999999999</v>
       </c>
       <c r="E6" s="0">
         <v>1.1910000000000001</v>
       </c>
       <c r="F6" s="0">
-        <v>0.56599999999999995</v>
+        <v>0.67800000000000005</v>
       </c>
       <c r="G6" s="0">
         <v>-0.63800000000000001</v>
@@ -234,19 +234,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>3.4239999999999999</v>
+        <v>7.2830000000000004</v>
       </c>
       <c r="C7" s="0">
-        <v>2.2360000000000002</v>
+        <v>2.96</v>
       </c>
       <c r="D7" s="0">
-        <v>1.117</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="E7" s="0">
         <v>1.2110000000000001</v>
       </c>
       <c r="F7" s="0">
-        <v>0.56299999999999994</v>
+        <v>0.54800000000000004</v>
       </c>
       <c r="G7" s="0">
         <v>-0.622</v>

</xml_diff>